<commit_message>
Classify rail transport VA codes as non-RTA
</commit_message>
<xml_diff>
--- a/docs/icd-causegrp-mappings/ICD-to-VA-Buckets/WHO_2022_VA_RTA_NonRTA_Review.xlsx
+++ b/docs/icd-causegrp-mappings/ICD-to-VA-Buckets/WHO_2022_VA_RTA_NonRTA_Review.xlsx
@@ -38846,22 +38846,18 @@
       </c>
       <c r="H710" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I710" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J710" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J710" t="inlineStr"/>
       <c r="K710" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L710" t="inlineStr"/>
@@ -38904,22 +38900,18 @@
       </c>
       <c r="H711" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I711" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J711" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J711" t="inlineStr"/>
       <c r="K711" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L711" t="inlineStr"/>
@@ -38962,22 +38954,18 @@
       </c>
       <c r="H712" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I712" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J712" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J712" t="inlineStr"/>
       <c r="K712" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L712" t="inlineStr"/>
@@ -39020,22 +39008,18 @@
       </c>
       <c r="H713" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I713" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J713" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J713" t="inlineStr"/>
       <c r="K713" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L713" t="inlineStr"/>
@@ -39078,22 +39062,18 @@
       </c>
       <c r="H714" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I714" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J714" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J714" t="inlineStr"/>
       <c r="K714" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L714" t="inlineStr"/>
@@ -39136,22 +39116,18 @@
       </c>
       <c r="H715" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I715" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J715" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J715" t="inlineStr"/>
       <c r="K715" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L715" t="inlineStr"/>
@@ -39194,22 +39170,18 @@
       </c>
       <c r="H716" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I716" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J716" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J716" t="inlineStr"/>
       <c r="K716" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L716" t="inlineStr"/>
@@ -39252,22 +39224,18 @@
       </c>
       <c r="H717" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I717" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J717" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J717" t="inlineStr"/>
       <c r="K717" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L717" t="inlineStr"/>
@@ -39472,22 +39440,18 @@
       </c>
       <c r="H721" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I721" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J721" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J721" t="inlineStr"/>
       <c r="K721" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L721" t="inlineStr"/>
@@ -39530,22 +39494,18 @@
       </c>
       <c r="H722" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I722" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J722" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J722" t="inlineStr"/>
       <c r="K722" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L722" t="inlineStr"/>
@@ -39588,22 +39548,18 @@
       </c>
       <c r="H723" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I723" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J723" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J723" t="inlineStr"/>
       <c r="K723" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L723" t="inlineStr"/>
@@ -39646,22 +39602,18 @@
       </c>
       <c r="H724" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I724" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J724" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J724" t="inlineStr"/>
       <c r="K724" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L724" t="inlineStr"/>
@@ -39704,22 +39656,18 @@
       </c>
       <c r="H725" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I725" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J725" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J725" t="inlineStr"/>
       <c r="K725" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L725" t="inlineStr"/>
@@ -39762,22 +39710,18 @@
       </c>
       <c r="H726" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I726" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J726" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J726" t="inlineStr"/>
       <c r="K726" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L726" t="inlineStr"/>
@@ -39820,22 +39764,18 @@
       </c>
       <c r="H727" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="I727" t="inlineStr">
         <is>
-          <t>Road traffic accident</t>
-        </is>
-      </c>
-      <c r="J727" t="inlineStr">
-        <is>
-          <t>Review: listed in footnote but title does not explicitly say traffic.</t>
-        </is>
-      </c>
+          <t>Other transport accident</t>
+        </is>
+      </c>
+      <c r="J727" t="inlineStr"/>
       <c r="K727" t="inlineStr">
         <is>
-          <t>VAs-12.01</t>
+          <t>VAs-12.02</t>
         </is>
       </c>
       <c r="L727" t="inlineStr"/>
@@ -49059,7 +48999,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>334</v>
+        <v>319</v>
       </c>
     </row>
     <row r="5">
@@ -49069,7 +49009,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>541</v>
+        <v>556</v>
       </c>
     </row>
     <row r="6">
@@ -49080,7 +49020,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Codes in RoadTraffic_Footnote are proposed as VAs-12.01 except V90-V99 and Y85.9, which are proposed as VAs-12.02. Review flags call out titles that do not explicitly say traffic.</t>
+          <t>Codes in RoadTraffic_Footnote are proposed as VAs-12.01 except V90-V99, Y85.9, and rail/streetcar events that do not explicitly say traffic accident; these are proposed as VAs-12.02. Review flags call out titles that do not explicitly say traffic.</t>
         </is>
       </c>
     </row>

</xml_diff>